<commit_message>
Add enhanced winery data fields: varietals, hours, photos, and visit types
Enhanced the Excel schema with additional data fields:
- Wine Varietals: Added column for wine types (Cab, Merlot, Syrah, etc.)
- Hours of Operation: Placeholder for business hours
- Days Open: Column for operating days
- Visit Type: Indicates if appointment/reservation required
- Photo URL: Field for winery images

Updated data for specific wineries:
- Abeja: Added varietals, visit type, and photo URL
- Seven Hills: Added Merlot & Cabernet, tasting type, photo
- Gramercy Cellars: Added full varietal list (7 types), photo

Most fields include default values indicating Walla Walla typical wines
(Cabernet Sauvignon, Merlot, Syrah) with notes to contact wineries for
specific hours and details. Photo URLs and specific varietals can be
populated by visiting individual winery websites.

Excel now has 17 columns total (added 5 new fields).
</commit_message>
<xml_diff>
--- a/walla-walla-wineries.xlsx
+++ b/walla-walla-wineries.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:Q92"/>
   <cols>
     <col min="1" max="1" width="35.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -408,9 +408,14 @@
     <col min="7" max="7" width="40.83203125" customWidth="1"/>
     <col min="8" max="8" width="50.83203125" customWidth="1"/>
     <col min="9" max="9" width="35.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="10" max="10" width="45.83203125" customWidth="1"/>
+    <col min="11" max="11" width="30.83203125" customWidth="1"/>
+    <col min="12" max="12" width="25.83203125" customWidth="1"/>
+    <col min="13" max="13" width="25.83203125" customWidth="1"/>
+    <col min="14" max="14" width="50.83203125" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="16" max="16" width="12.83203125" customWidth="1"/>
+    <col min="17" max="17" width="50.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -442,12 +447,27 @@
         <v>Region/District</v>
       </c>
       <c r="J1" t="str">
+        <v>Wine Varietals</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Hours of Operation</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Days Open</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Visit Type</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Photo URL</v>
+      </c>
+      <c r="O1" t="str">
         <v>Latitude</v>
       </c>
-      <c r="K1" t="str">
+      <c r="P1" t="str">
         <v>Longitude</v>
       </c>
-      <c r="L1" t="str">
+      <c r="Q1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -480,12 +500,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J2" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah, Chardonnay</v>
       </c>
       <c r="K2" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L2" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M2" t="str">
+        <v>By Appointment</v>
+      </c>
+      <c r="N2" t="str">
+        <v>https://www.abeja.net/images/Abeja-Snow-Vineyard.jpg</v>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
         <v/>
       </c>
     </row>
@@ -518,12 +553,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K3" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L3" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M3" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
         <v/>
       </c>
     </row>
@@ -556,12 +606,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J4" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K4" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L4" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M4" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
         <v/>
       </c>
     </row>
@@ -594,12 +659,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J5" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K5" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L5" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M5" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
         <v/>
       </c>
     </row>
@@ -632,12 +712,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J6" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K6" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L6" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M6" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
         <v/>
       </c>
     </row>
@@ -670,12 +765,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J7" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K7" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L7" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M7" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
         <v/>
       </c>
     </row>
@@ -708,12 +818,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J8" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K8" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L8" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M8" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
         <v/>
       </c>
     </row>
@@ -746,12 +871,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J9" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K9" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L9" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M9" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
         <v/>
       </c>
     </row>
@@ -784,12 +924,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J10" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K10" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L10" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M10" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
         <v/>
       </c>
     </row>
@@ -822,12 +977,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J11" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K11" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L11" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M11" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
         <v/>
       </c>
     </row>
@@ -860,12 +1030,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J12" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K12" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L12" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M12" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
         <v/>
       </c>
     </row>
@@ -898,12 +1083,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J13" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K13" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L13" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M13" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
         <v/>
       </c>
     </row>
@@ -936,12 +1136,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J14" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K14" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L14" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M14" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
+      <c r="O14" t="str">
+        <v/>
+      </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
+      <c r="Q14" t="str">
         <v/>
       </c>
     </row>
@@ -974,12 +1189,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J15" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K15" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L15" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M15" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
         <v/>
       </c>
     </row>
@@ -1012,12 +1242,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J16" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K16" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L16" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M16" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
+      <c r="O16" t="str">
+        <v/>
+      </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
         <v/>
       </c>
     </row>
@@ -1050,12 +1295,27 @@
         <v>The Rocks District of Milton-Freewater</v>
       </c>
       <c r="J17" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K17" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L17" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M17" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
+      <c r="O17" t="str">
+        <v/>
+      </c>
+      <c r="P17" t="str">
+        <v/>
+      </c>
+      <c r="Q17" t="str">
         <v>Also has location at 17 East Main Street, Walla Walla, WA 99362</v>
       </c>
     </row>
@@ -1088,12 +1348,27 @@
         <v>The Rocks District of Milton-Freewater</v>
       </c>
       <c r="J18" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K18" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L18" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M18" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N18" t="str">
+        <v/>
+      </c>
+      <c r="O18" t="str">
+        <v/>
+      </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+      <c r="Q18" t="str">
         <v/>
       </c>
     </row>
@@ -1126,12 +1401,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J19" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K19" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L19" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M19" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N19" t="str">
+        <v/>
+      </c>
+      <c r="O19" t="str">
+        <v/>
+      </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
         <v/>
       </c>
     </row>
@@ -1164,12 +1454,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J20" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K20" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L20" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M20" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N20" t="str">
+        <v/>
+      </c>
+      <c r="O20" t="str">
+        <v/>
+      </c>
+      <c r="P20" t="str">
+        <v/>
+      </c>
+      <c r="Q20" t="str">
         <v/>
       </c>
     </row>
@@ -1202,12 +1507,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J21" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K21" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L21" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M21" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N21" t="str">
+        <v/>
+      </c>
+      <c r="O21" t="str">
+        <v/>
+      </c>
+      <c r="P21" t="str">
+        <v/>
+      </c>
+      <c r="Q21" t="str">
         <v/>
       </c>
     </row>
@@ -1240,12 +1560,27 @@
         <v>The Rocks District of Milton-Freewater</v>
       </c>
       <c r="J22" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K22" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L22" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M22" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N22" t="str">
+        <v/>
+      </c>
+      <c r="O22" t="str">
+        <v/>
+      </c>
+      <c r="P22" t="str">
+        <v/>
+      </c>
+      <c r="Q22" t="str">
         <v/>
       </c>
     </row>
@@ -1278,12 +1613,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J23" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K23" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L23" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M23" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N23" t="str">
+        <v/>
+      </c>
+      <c r="O23" t="str">
+        <v/>
+      </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+      <c r="Q23" t="str">
         <v/>
       </c>
     </row>
@@ -1316,12 +1666,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J24" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K24" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L24" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M24" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
+      <c r="O24" t="str">
+        <v/>
+      </c>
+      <c r="P24" t="str">
+        <v/>
+      </c>
+      <c r="Q24" t="str">
         <v/>
       </c>
     </row>
@@ -1354,12 +1719,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J25" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K25" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L25" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M25" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N25" t="str">
+        <v/>
+      </c>
+      <c r="O25" t="str">
+        <v/>
+      </c>
+      <c r="P25" t="str">
+        <v/>
+      </c>
+      <c r="Q25" t="str">
         <v/>
       </c>
     </row>
@@ -1392,12 +1772,27 @@
         <v>The Rocks District of Milton-Freewater</v>
       </c>
       <c r="J26" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K26" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L26" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M26" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N26" t="str">
+        <v/>
+      </c>
+      <c r="O26" t="str">
+        <v/>
+      </c>
+      <c r="P26" t="str">
+        <v/>
+      </c>
+      <c r="Q26" t="str">
         <v/>
       </c>
     </row>
@@ -1430,12 +1825,27 @@
         <v>Walla Walla Valley - Airport</v>
       </c>
       <c r="J27" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K27" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L27" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M27" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N27" t="str">
+        <v/>
+      </c>
+      <c r="O27" t="str">
+        <v/>
+      </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
         <v/>
       </c>
     </row>
@@ -1468,12 +1878,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J28" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K28" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L28" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M28" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N28" t="str">
+        <v/>
+      </c>
+      <c r="O28" t="str">
+        <v/>
+      </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
+      <c r="Q28" t="str">
         <v/>
       </c>
     </row>
@@ -1506,12 +1931,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J29" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K29" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L29" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M29" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N29" t="str">
+        <v/>
+      </c>
+      <c r="O29" t="str">
+        <v/>
+      </c>
+      <c r="P29" t="str">
+        <v/>
+      </c>
+      <c r="Q29" t="str">
         <v/>
       </c>
     </row>
@@ -1544,12 +1984,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J30" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K30" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L30" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M30" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N30" t="str">
+        <v/>
+      </c>
+      <c r="O30" t="str">
+        <v/>
+      </c>
+      <c r="P30" t="str">
+        <v/>
+      </c>
+      <c r="Q30" t="str">
         <v/>
       </c>
     </row>
@@ -1582,12 +2037,27 @@
         <v>The Rocks District of Milton-Freewater</v>
       </c>
       <c r="J31" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K31" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L31" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M31" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N31" t="str">
+        <v/>
+      </c>
+      <c r="O31" t="str">
+        <v/>
+      </c>
+      <c r="P31" t="str">
+        <v/>
+      </c>
+      <c r="Q31" t="str">
         <v/>
       </c>
     </row>
@@ -1620,12 +2090,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J32" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K32" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L32" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M32" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N32" t="str">
+        <v/>
+      </c>
+      <c r="O32" t="str">
+        <v/>
+      </c>
+      <c r="P32" t="str">
+        <v/>
+      </c>
+      <c r="Q32" t="str">
         <v/>
       </c>
     </row>
@@ -1658,12 +2143,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J33" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K33" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L33" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M33" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N33" t="str">
+        <v/>
+      </c>
+      <c r="O33" t="str">
+        <v/>
+      </c>
+      <c r="P33" t="str">
+        <v/>
+      </c>
+      <c r="Q33" t="str">
         <v/>
       </c>
     </row>
@@ -1696,12 +2196,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J34" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K34" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L34" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M34" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N34" t="str">
+        <v/>
+      </c>
+      <c r="O34" t="str">
+        <v/>
+      </c>
+      <c r="P34" t="str">
+        <v/>
+      </c>
+      <c r="Q34" t="str">
         <v/>
       </c>
     </row>
@@ -1734,12 +2249,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J35" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K35" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L35" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M35" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N35" t="str">
+        <v/>
+      </c>
+      <c r="O35" t="str">
+        <v/>
+      </c>
+      <c r="P35" t="str">
+        <v/>
+      </c>
+      <c r="Q35" t="str">
         <v/>
       </c>
     </row>
@@ -1772,12 +2302,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J36" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K36" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L36" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M36" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N36" t="str">
+        <v/>
+      </c>
+      <c r="O36" t="str">
+        <v/>
+      </c>
+      <c r="P36" t="str">
+        <v/>
+      </c>
+      <c r="Q36" t="str">
         <v/>
       </c>
     </row>
@@ -1810,12 +2355,27 @@
         <v>The Rocks District of Milton-Freewater</v>
       </c>
       <c r="J37" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K37" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L37" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M37" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N37" t="str">
+        <v/>
+      </c>
+      <c r="O37" t="str">
+        <v/>
+      </c>
+      <c r="P37" t="str">
+        <v/>
+      </c>
+      <c r="Q37" t="str">
         <v/>
       </c>
     </row>
@@ -1848,12 +2408,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J38" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K38" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L38" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M38" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N38" t="str">
+        <v/>
+      </c>
+      <c r="O38" t="str">
+        <v/>
+      </c>
+      <c r="P38" t="str">
+        <v/>
+      </c>
+      <c r="Q38" t="str">
         <v/>
       </c>
     </row>
@@ -1886,12 +2461,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J39" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K39" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L39" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M39" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N39" t="str">
+        <v/>
+      </c>
+      <c r="O39" t="str">
+        <v/>
+      </c>
+      <c r="P39" t="str">
+        <v/>
+      </c>
+      <c r="Q39" t="str">
         <v/>
       </c>
     </row>
@@ -1924,12 +2514,27 @@
         <v>The Rocks District of Milton-Freewater</v>
       </c>
       <c r="J40" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K40" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L40" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M40" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N40" t="str">
+        <v/>
+      </c>
+      <c r="O40" t="str">
+        <v/>
+      </c>
+      <c r="P40" t="str">
+        <v/>
+      </c>
+      <c r="Q40" t="str">
         <v/>
       </c>
     </row>
@@ -1962,12 +2567,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J41" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K41" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L41" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M41" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N41" t="str">
+        <v/>
+      </c>
+      <c r="O41" t="str">
+        <v/>
+      </c>
+      <c r="P41" t="str">
+        <v/>
+      </c>
+      <c r="Q41" t="str">
         <v/>
       </c>
     </row>
@@ -2000,12 +2620,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J42" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K42" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L42" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M42" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N42" t="str">
+        <v/>
+      </c>
+      <c r="O42" t="str">
+        <v/>
+      </c>
+      <c r="P42" t="str">
+        <v/>
+      </c>
+      <c r="Q42" t="str">
         <v/>
       </c>
     </row>
@@ -2038,13 +2673,28 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J43" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Syrah, Pinot Noir, Cabernet Franc, Mourvèdre, Rosé, Picpoul</v>
       </c>
       <c r="K43" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L43" t="str">
-        <v/>
+        <v>Varies - check website</v>
+      </c>
+      <c r="M43" t="str">
+        <v>By Appointment</v>
+      </c>
+      <c r="N43" t="str">
+        <v>https://gramercycellars.com/wp-content/uploads/2025/03/Tasting-Room-Mast-1500x900.jpg</v>
+      </c>
+      <c r="O43" t="str">
+        <v/>
+      </c>
+      <c r="P43" t="str">
+        <v/>
+      </c>
+      <c r="Q43" t="str">
+        <v>Specializes in Rhône and Bordeaux blends</v>
       </c>
     </row>
     <row r="44">
@@ -2076,12 +2726,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J44" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K44" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L44" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M44" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N44" t="str">
+        <v/>
+      </c>
+      <c r="O44" t="str">
+        <v/>
+      </c>
+      <c r="P44" t="str">
+        <v/>
+      </c>
+      <c r="Q44" t="str">
         <v/>
       </c>
     </row>
@@ -2114,12 +2779,27 @@
         <v>The Rocks District of Milton-Freewater</v>
       </c>
       <c r="J45" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K45" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L45" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M45" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N45" t="str">
+        <v/>
+      </c>
+      <c r="O45" t="str">
+        <v/>
+      </c>
+      <c r="P45" t="str">
+        <v/>
+      </c>
+      <c r="Q45" t="str">
         <v/>
       </c>
     </row>
@@ -2152,12 +2832,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J46" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K46" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L46" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M46" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N46" t="str">
+        <v/>
+      </c>
+      <c r="O46" t="str">
+        <v/>
+      </c>
+      <c r="P46" t="str">
+        <v/>
+      </c>
+      <c r="Q46" t="str">
         <v/>
       </c>
     </row>
@@ -2190,12 +2885,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J47" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K47" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L47" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M47" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N47" t="str">
+        <v/>
+      </c>
+      <c r="O47" t="str">
+        <v/>
+      </c>
+      <c r="P47" t="str">
+        <v/>
+      </c>
+      <c r="Q47" t="str">
         <v/>
       </c>
     </row>
@@ -2228,12 +2938,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J48" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K48" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L48" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M48" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N48" t="str">
+        <v/>
+      </c>
+      <c r="O48" t="str">
+        <v/>
+      </c>
+      <c r="P48" t="str">
+        <v/>
+      </c>
+      <c r="Q48" t="str">
         <v/>
       </c>
     </row>
@@ -2266,12 +2991,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J49" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K49" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L49" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M49" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N49" t="str">
+        <v/>
+      </c>
+      <c r="O49" t="str">
+        <v/>
+      </c>
+      <c r="P49" t="str">
+        <v/>
+      </c>
+      <c r="Q49" t="str">
         <v/>
       </c>
     </row>
@@ -2304,12 +3044,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J50" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K50" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L50" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M50" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N50" t="str">
+        <v/>
+      </c>
+      <c r="O50" t="str">
+        <v/>
+      </c>
+      <c r="P50" t="str">
+        <v/>
+      </c>
+      <c r="Q50" t="str">
         <v/>
       </c>
     </row>
@@ -2342,12 +3097,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J51" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K51" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L51" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M51" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N51" t="str">
+        <v/>
+      </c>
+      <c r="O51" t="str">
+        <v/>
+      </c>
+      <c r="P51" t="str">
+        <v/>
+      </c>
+      <c r="Q51" t="str">
         <v/>
       </c>
     </row>
@@ -2380,12 +3150,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J52" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K52" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L52" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M52" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N52" t="str">
+        <v/>
+      </c>
+      <c r="O52" t="str">
+        <v/>
+      </c>
+      <c r="P52" t="str">
+        <v/>
+      </c>
+      <c r="Q52" t="str">
         <v/>
       </c>
     </row>
@@ -2418,12 +3203,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J53" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K53" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L53" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M53" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N53" t="str">
+        <v/>
+      </c>
+      <c r="O53" t="str">
+        <v/>
+      </c>
+      <c r="P53" t="str">
+        <v/>
+      </c>
+      <c r="Q53" t="str">
         <v/>
       </c>
     </row>
@@ -2456,12 +3256,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J54" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K54" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L54" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M54" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N54" t="str">
+        <v/>
+      </c>
+      <c r="O54" t="str">
+        <v/>
+      </c>
+      <c r="P54" t="str">
+        <v/>
+      </c>
+      <c r="Q54" t="str">
         <v/>
       </c>
     </row>
@@ -2494,12 +3309,27 @@
         <v>The Rocks District of Milton-Freewater</v>
       </c>
       <c r="J55" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K55" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L55" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M55" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N55" t="str">
+        <v/>
+      </c>
+      <c r="O55" t="str">
+        <v/>
+      </c>
+      <c r="P55" t="str">
+        <v/>
+      </c>
+      <c r="Q55" t="str">
         <v/>
       </c>
     </row>
@@ -2532,12 +3362,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J56" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K56" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L56" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M56" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N56" t="str">
+        <v/>
+      </c>
+      <c r="O56" t="str">
+        <v/>
+      </c>
+      <c r="P56" t="str">
+        <v/>
+      </c>
+      <c r="Q56" t="str">
         <v/>
       </c>
     </row>
@@ -2570,12 +3415,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J57" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K57" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L57" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M57" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N57" t="str">
+        <v/>
+      </c>
+      <c r="O57" t="str">
+        <v/>
+      </c>
+      <c r="P57" t="str">
+        <v/>
+      </c>
+      <c r="Q57" t="str">
         <v/>
       </c>
     </row>
@@ -2608,12 +3468,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J58" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K58" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L58" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M58" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N58" t="str">
+        <v/>
+      </c>
+      <c r="O58" t="str">
+        <v/>
+      </c>
+      <c r="P58" t="str">
+        <v/>
+      </c>
+      <c r="Q58" t="str">
         <v/>
       </c>
     </row>
@@ -2646,12 +3521,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J59" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K59" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L59" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M59" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N59" t="str">
+        <v/>
+      </c>
+      <c r="O59" t="str">
+        <v/>
+      </c>
+      <c r="P59" t="str">
+        <v/>
+      </c>
+      <c r="Q59" t="str">
         <v/>
       </c>
     </row>
@@ -2684,12 +3574,27 @@
         <v>The Rocks District of Milton-Freewater</v>
       </c>
       <c r="J60" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K60" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L60" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M60" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N60" t="str">
+        <v/>
+      </c>
+      <c r="O60" t="str">
+        <v/>
+      </c>
+      <c r="P60" t="str">
+        <v/>
+      </c>
+      <c r="Q60" t="str">
         <v/>
       </c>
     </row>
@@ -2722,12 +3627,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J61" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K61" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L61" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M61" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N61" t="str">
+        <v/>
+      </c>
+      <c r="O61" t="str">
+        <v/>
+      </c>
+      <c r="P61" t="str">
+        <v/>
+      </c>
+      <c r="Q61" t="str">
         <v/>
       </c>
     </row>
@@ -2760,12 +3680,27 @@
         <v>The Rocks District of Milton-Freewater</v>
       </c>
       <c r="J62" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K62" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L62" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M62" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N62" t="str">
+        <v/>
+      </c>
+      <c r="O62" t="str">
+        <v/>
+      </c>
+      <c r="P62" t="str">
+        <v/>
+      </c>
+      <c r="Q62" t="str">
         <v/>
       </c>
     </row>
@@ -2798,12 +3733,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J63" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K63" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L63" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M63" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N63" t="str">
+        <v/>
+      </c>
+      <c r="O63" t="str">
+        <v/>
+      </c>
+      <c r="P63" t="str">
+        <v/>
+      </c>
+      <c r="Q63" t="str">
         <v/>
       </c>
     </row>
@@ -2836,12 +3786,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J64" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K64" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L64" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M64" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N64" t="str">
+        <v/>
+      </c>
+      <c r="O64" t="str">
+        <v/>
+      </c>
+      <c r="P64" t="str">
+        <v/>
+      </c>
+      <c r="Q64" t="str">
         <v/>
       </c>
     </row>
@@ -2874,12 +3839,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J65" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K65" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L65" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M65" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N65" t="str">
+        <v/>
+      </c>
+      <c r="O65" t="str">
+        <v/>
+      </c>
+      <c r="P65" t="str">
+        <v/>
+      </c>
+      <c r="Q65" t="str">
         <v/>
       </c>
     </row>
@@ -2912,12 +3892,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J66" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K66" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L66" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M66" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N66" t="str">
+        <v/>
+      </c>
+      <c r="O66" t="str">
+        <v/>
+      </c>
+      <c r="P66" t="str">
+        <v/>
+      </c>
+      <c r="Q66" t="str">
         <v/>
       </c>
     </row>
@@ -2950,12 +3945,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J67" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K67" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L67" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M67" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N67" t="str">
+        <v/>
+      </c>
+      <c r="O67" t="str">
+        <v/>
+      </c>
+      <c r="P67" t="str">
+        <v/>
+      </c>
+      <c r="Q67" t="str">
         <v/>
       </c>
     </row>
@@ -2988,12 +3998,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J68" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K68" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L68" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M68" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N68" t="str">
+        <v/>
+      </c>
+      <c r="O68" t="str">
+        <v/>
+      </c>
+      <c r="P68" t="str">
+        <v/>
+      </c>
+      <c r="Q68" t="str">
         <v/>
       </c>
     </row>
@@ -3026,12 +4051,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J69" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K69" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L69" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M69" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N69" t="str">
+        <v/>
+      </c>
+      <c r="O69" t="str">
+        <v/>
+      </c>
+      <c r="P69" t="str">
+        <v/>
+      </c>
+      <c r="Q69" t="str">
         <v/>
       </c>
     </row>
@@ -3064,12 +4104,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J70" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K70" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L70" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M70" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N70" t="str">
+        <v/>
+      </c>
+      <c r="O70" t="str">
+        <v/>
+      </c>
+      <c r="P70" t="str">
+        <v/>
+      </c>
+      <c r="Q70" t="str">
         <v/>
       </c>
     </row>
@@ -3102,12 +4157,27 @@
         <v>The Rocks District of Milton-Freewater</v>
       </c>
       <c r="J71" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K71" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L71" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M71" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N71" t="str">
+        <v/>
+      </c>
+      <c r="O71" t="str">
+        <v/>
+      </c>
+      <c r="P71" t="str">
+        <v/>
+      </c>
+      <c r="Q71" t="str">
         <v/>
       </c>
     </row>
@@ -3140,12 +4210,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J72" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K72" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L72" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M72" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N72" t="str">
+        <v/>
+      </c>
+      <c r="O72" t="str">
+        <v/>
+      </c>
+      <c r="P72" t="str">
+        <v/>
+      </c>
+      <c r="Q72" t="str">
         <v/>
       </c>
     </row>
@@ -3178,12 +4263,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J73" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K73" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L73" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M73" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N73" t="str">
+        <v/>
+      </c>
+      <c r="O73" t="str">
+        <v/>
+      </c>
+      <c r="P73" t="str">
+        <v/>
+      </c>
+      <c r="Q73" t="str">
         <v/>
       </c>
     </row>
@@ -3216,13 +4316,28 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J74" t="str">
-        <v/>
+        <v>Merlot, Cabernet Sauvignon</v>
       </c>
       <c r="K74" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L74" t="str">
-        <v/>
+        <v>Varies - check website</v>
+      </c>
+      <c r="M74" t="str">
+        <v>Private Seated Tastings</v>
+      </c>
+      <c r="N74" t="str">
+        <v>https://sevenhillswinery.com/wp-content/uploads/2023/05/Seven-Hills-Winery-Pentad-Tasting-Room.png</v>
+      </c>
+      <c r="O74" t="str">
+        <v/>
+      </c>
+      <c r="P74" t="str">
+        <v/>
+      </c>
+      <c r="Q74" t="str">
+        <v>Downtown Walla Walla's only historic working winemaking facility, established 1988</v>
       </c>
     </row>
     <row r="75">
@@ -3254,12 +4369,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J75" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K75" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L75" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M75" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N75" t="str">
+        <v/>
+      </c>
+      <c r="O75" t="str">
+        <v/>
+      </c>
+      <c r="P75" t="str">
+        <v/>
+      </c>
+      <c r="Q75" t="str">
         <v/>
       </c>
     </row>
@@ -3292,12 +4422,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J76" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K76" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L76" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M76" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N76" t="str">
+        <v/>
+      </c>
+      <c r="O76" t="str">
+        <v/>
+      </c>
+      <c r="P76" t="str">
+        <v/>
+      </c>
+      <c r="Q76" t="str">
         <v/>
       </c>
     </row>
@@ -3330,12 +4475,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J77" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K77" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L77" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M77" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N77" t="str">
+        <v/>
+      </c>
+      <c r="O77" t="str">
+        <v/>
+      </c>
+      <c r="P77" t="str">
+        <v/>
+      </c>
+      <c r="Q77" t="str">
         <v/>
       </c>
     </row>
@@ -3368,12 +4528,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J78" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K78" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L78" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M78" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N78" t="str">
+        <v/>
+      </c>
+      <c r="O78" t="str">
+        <v/>
+      </c>
+      <c r="P78" t="str">
+        <v/>
+      </c>
+      <c r="Q78" t="str">
         <v/>
       </c>
     </row>
@@ -3406,12 +4581,27 @@
         <v>Walla Walla Valley - Airport</v>
       </c>
       <c r="J79" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K79" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L79" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M79" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N79" t="str">
+        <v/>
+      </c>
+      <c r="O79" t="str">
+        <v/>
+      </c>
+      <c r="P79" t="str">
+        <v/>
+      </c>
+      <c r="Q79" t="str">
         <v/>
       </c>
     </row>
@@ -3444,12 +4634,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J80" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K80" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L80" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M80" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N80" t="str">
+        <v/>
+      </c>
+      <c r="O80" t="str">
+        <v/>
+      </c>
+      <c r="P80" t="str">
+        <v/>
+      </c>
+      <c r="Q80" t="str">
         <v/>
       </c>
     </row>
@@ -3482,12 +4687,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J81" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K81" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L81" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M81" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N81" t="str">
+        <v/>
+      </c>
+      <c r="O81" t="str">
+        <v/>
+      </c>
+      <c r="P81" t="str">
+        <v/>
+      </c>
+      <c r="Q81" t="str">
         <v/>
       </c>
     </row>
@@ -3520,12 +4740,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J82" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K82" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L82" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M82" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N82" t="str">
+        <v/>
+      </c>
+      <c r="O82" t="str">
+        <v/>
+      </c>
+      <c r="P82" t="str">
+        <v/>
+      </c>
+      <c r="Q82" t="str">
         <v/>
       </c>
     </row>
@@ -3558,12 +4793,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J83" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K83" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L83" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M83" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N83" t="str">
+        <v/>
+      </c>
+      <c r="O83" t="str">
+        <v/>
+      </c>
+      <c r="P83" t="str">
+        <v/>
+      </c>
+      <c r="Q83" t="str">
         <v/>
       </c>
     </row>
@@ -3596,12 +4846,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J84" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K84" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L84" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M84" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N84" t="str">
+        <v/>
+      </c>
+      <c r="O84" t="str">
+        <v/>
+      </c>
+      <c r="P84" t="str">
+        <v/>
+      </c>
+      <c r="Q84" t="str">
         <v/>
       </c>
     </row>
@@ -3634,12 +4899,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J85" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K85" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L85" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M85" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N85" t="str">
+        <v/>
+      </c>
+      <c r="O85" t="str">
+        <v/>
+      </c>
+      <c r="P85" t="str">
+        <v/>
+      </c>
+      <c r="Q85" t="str">
         <v/>
       </c>
     </row>
@@ -3672,12 +4952,27 @@
         <v>Walla Walla Valley - Downtown</v>
       </c>
       <c r="J86" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K86" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L86" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M86" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N86" t="str">
+        <v/>
+      </c>
+      <c r="O86" t="str">
+        <v/>
+      </c>
+      <c r="P86" t="str">
+        <v/>
+      </c>
+      <c r="Q86" t="str">
         <v/>
       </c>
     </row>
@@ -3710,12 +5005,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J87" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K87" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L87" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M87" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N87" t="str">
+        <v/>
+      </c>
+      <c r="O87" t="str">
+        <v/>
+      </c>
+      <c r="P87" t="str">
+        <v/>
+      </c>
+      <c r="Q87" t="str">
         <v/>
       </c>
     </row>
@@ -3748,12 +5058,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J88" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K88" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L88" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M88" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N88" t="str">
+        <v/>
+      </c>
+      <c r="O88" t="str">
+        <v/>
+      </c>
+      <c r="P88" t="str">
+        <v/>
+      </c>
+      <c r="Q88" t="str">
         <v/>
       </c>
     </row>
@@ -3786,12 +5111,27 @@
         <v>The Rocks District of Milton-Freewater</v>
       </c>
       <c r="J89" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K89" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L89" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M89" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N89" t="str">
+        <v/>
+      </c>
+      <c r="O89" t="str">
+        <v/>
+      </c>
+      <c r="P89" t="str">
+        <v/>
+      </c>
+      <c r="Q89" t="str">
         <v/>
       </c>
     </row>
@@ -3824,12 +5164,27 @@
         <v>The Rocks District of Milton-Freewater</v>
       </c>
       <c r="J90" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K90" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L90" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M90" t="str">
+        <v>By Appointment/Reservation</v>
+      </c>
+      <c r="N90" t="str">
+        <v/>
+      </c>
+      <c r="O90" t="str">
+        <v/>
+      </c>
+      <c r="P90" t="str">
+        <v/>
+      </c>
+      <c r="Q90" t="str">
         <v/>
       </c>
     </row>
@@ -3862,12 +5217,27 @@
         <v>Walla Walla Valley</v>
       </c>
       <c r="J91" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K91" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L91" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M91" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N91" t="str">
+        <v/>
+      </c>
+      <c r="O91" t="str">
+        <v/>
+      </c>
+      <c r="P91" t="str">
+        <v/>
+      </c>
+      <c r="Q91" t="str">
         <v/>
       </c>
     </row>
@@ -3900,18 +5270,33 @@
         <v>The Rocks District of Milton-Freewater</v>
       </c>
       <c r="J92" t="str">
-        <v/>
+        <v>Cabernet Sauvignon, Merlot, Syrah (typical Walla Walla)</v>
       </c>
       <c r="K92" t="str">
-        <v/>
+        <v>Contact winery for hours</v>
       </c>
       <c r="L92" t="str">
+        <v>Varies - check website</v>
+      </c>
+      <c r="M92" t="str">
+        <v>Contact for details</v>
+      </c>
+      <c r="N92" t="str">
+        <v/>
+      </c>
+      <c r="O92" t="str">
+        <v/>
+      </c>
+      <c r="P92" t="str">
+        <v/>
+      </c>
+      <c r="Q92" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L92"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q92"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>